<commit_message>
Fix objetivo: precio real Cerdo Blanco de Lleida (no equivalente) + aclarar centimos
</commit_message>
<xml_diff>
--- a/data/master.xlsx
+++ b/data/master.xlsx
@@ -72,7 +72,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -117,6 +117,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FCE4D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9E8F5"/>
       </patternFill>
     </fill>
   </fills>
@@ -194,7 +199,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="165" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
@@ -280,6 +285,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2410,8 +2418,8 @@
       <c r="Q36" s="21" t="n">
         <v>1.815</v>
       </c>
-      <c r="R36" s="22" t="n">
-        <v>1.31</v>
+      <c r="R36" s="31" t="n">
+        <v>1.3</v>
       </c>
     </row>
     <row r="37">
@@ -2466,8 +2474,8 @@
       <c r="Q37" s="21" t="n">
         <v>1.815</v>
       </c>
-      <c r="R37" s="22" t="n">
-        <v>1.3</v>
+      <c r="R37" s="31" t="n">
+        <v>1.29</v>
       </c>
     </row>
     <row r="38">
@@ -2522,8 +2530,8 @@
       <c r="Q38" s="21" t="n">
         <v>1.795</v>
       </c>
-      <c r="R38" s="22" t="n">
-        <v>1.29</v>
+      <c r="R38" s="31" t="n">
+        <v>1.285</v>
       </c>
     </row>
     <row r="39">
@@ -2578,8 +2586,8 @@
       <c r="Q39" s="21" t="n">
         <v>1.778</v>
       </c>
-      <c r="R39" s="22" t="n">
-        <v>1.29</v>
+      <c r="R39" s="31" t="n">
+        <v>1.285</v>
       </c>
     </row>
     <row r="40">
@@ -2634,8 +2642,8 @@
       <c r="Q40" s="21" t="n">
         <v>1.758</v>
       </c>
-      <c r="R40" s="22" t="n">
-        <v>1.29</v>
+      <c r="R40" s="31" t="n">
+        <v>1.295</v>
       </c>
     </row>
     <row r="41">
@@ -2690,8 +2698,8 @@
       <c r="Q41" s="21" t="n">
         <v>1.73</v>
       </c>
-      <c r="R41" s="22" t="n">
-        <v>1.3</v>
+      <c r="R41" s="31" t="n">
+        <v>1.325</v>
       </c>
     </row>
     <row r="42">
@@ -2746,8 +2754,8 @@
       <c r="Q42" s="21" t="n">
         <v>1.701</v>
       </c>
-      <c r="R42" s="22" t="n">
-        <v>1.33</v>
+      <c r="R42" s="31" t="n">
+        <v>1.35</v>
       </c>
     </row>
     <row r="43">
@@ -2802,8 +2810,8 @@
       <c r="Q43" s="21" t="n">
         <v>1.671</v>
       </c>
-      <c r="R43" s="22" t="n">
-        <v>1.35</v>
+      <c r="R43" s="31" t="n">
+        <v>1.36</v>
       </c>
     </row>
     <row r="44">
@@ -2858,8 +2866,8 @@
       <c r="Q44" s="21" t="n">
         <v>1.643</v>
       </c>
-      <c r="R44" s="22" t="n">
-        <v>1.36</v>
+      <c r="R44" s="31" t="n">
+        <v>1.363</v>
       </c>
     </row>
     <row r="45">
@@ -2914,8 +2922,8 @@
       <c r="Q45" s="21" t="n">
         <v>1.617</v>
       </c>
-      <c r="R45" s="22" t="n">
-        <v>1.36</v>
+      <c r="R45" s="31" t="n">
+        <v>1.365</v>
       </c>
     </row>
     <row r="46">
@@ -2970,8 +2978,8 @@
       <c r="Q46" s="21" t="n">
         <v>1.587</v>
       </c>
-      <c r="R46" s="22" t="n">
-        <v>1.37</v>
+      <c r="R46" s="31" t="n">
+        <v>1.34</v>
       </c>
     </row>
     <row r="47">

</xml_diff>

<commit_message>
Semana 39 procesada (real 1,315, acierto 1,1 cts) + bot revisa 3 veces/dia L-V
</commit_message>
<xml_diff>
--- a/data/master.xlsx
+++ b/data/master.xlsx
@@ -3034,7 +3034,9 @@
       <c r="Q47" s="21" t="n">
         <v>1.552</v>
       </c>
-      <c r="R47" s="21" t="n"/>
+      <c r="R47" s="22" t="n">
+        <v>1.315</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="1" t="n">

</xml_diff>

<commit_message>
PRIMERA VALIDACION EN VIVO: sem40 real 1.295 vs prediccion 1.283 = 1.2 cts de error (bate al naive de 2.0 cts)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/master.xlsx
+++ b/data/master.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="3" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="CEBADO LLEIDA" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="ALEMANIA" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="FRANCIA" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="DINAMARCA" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CEBADO LLEIDA" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ALEMANIA" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FRANCIA" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DINAMARCA" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="145621" fullCalcOnLoad="1"/>
@@ -299,7 +299,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor editAs="oneCell">
     <from>
       <col>0</col>
@@ -317,26 +317,26 @@
       <nvPicPr>
         <cNvPr id="2" name="1 Imagen"/>
         <cNvPicPr>
-          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1" noChangeArrowheads="1"/>
         </cNvPicPr>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId1"/>
-        <a:srcRect/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:srcRect xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr bwMode="auto">
-        <a:xfrm>
+        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:off x="464691" y="60960"/>
           <a:ext cx="1646177" cy="487680"/>
         </a:xfrm>
-        <a:prstGeom prst="rect">
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
           <avLst/>
         </a:prstGeom>
-        <a:noFill/>
-        <a:ln>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -348,7 +348,7 @@
 </file>
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor editAs="oneCell">
     <from>
       <col>0</col>
@@ -366,26 +366,26 @@
       <nvPicPr>
         <cNvPr id="2" name="1 Imagen"/>
         <cNvPicPr>
-          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1" noChangeArrowheads="1"/>
         </cNvPicPr>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId1"/>
-        <a:srcRect/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:srcRect xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr bwMode="auto">
-        <a:xfrm>
+        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:off x="478979" y="60960"/>
           <a:ext cx="1646177" cy="487680"/>
         </a:xfrm>
-        <a:prstGeom prst="rect">
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
           <avLst/>
         </a:prstGeom>
-        <a:noFill/>
-        <a:ln>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -397,7 +397,7 @@
 </file>
 
 <file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor editAs="oneCell">
     <from>
       <col>0</col>
@@ -415,26 +415,26 @@
       <nvPicPr>
         <cNvPr id="2" name="1 Imagen"/>
         <cNvPicPr>
-          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1" noChangeArrowheads="1"/>
         </cNvPicPr>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId1"/>
-        <a:srcRect/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:srcRect xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr bwMode="auto">
-        <a:xfrm>
+        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:off x="478979" y="60960"/>
           <a:ext cx="1646177" cy="487680"/>
         </a:xfrm>
-        <a:prstGeom prst="rect">
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
           <avLst/>
         </a:prstGeom>
-        <a:noFill/>
-        <a:ln>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -446,7 +446,7 @@
 </file>
 
 <file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor editAs="oneCell">
     <from>
       <col>0</col>
@@ -464,26 +464,26 @@
       <nvPicPr>
         <cNvPr id="2" name="1 Imagen"/>
         <cNvPicPr>
-          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1" noChangeArrowheads="1"/>
         </cNvPicPr>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId1"/>
-        <a:srcRect/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:srcRect xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr bwMode="auto">
-        <a:xfrm>
+        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:off x="478979" y="60960"/>
           <a:ext cx="1646177" cy="487680"/>
         </a:xfrm>
-        <a:prstGeom prst="rect">
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
           <avLst/>
         </a:prstGeom>
-        <a:noFill/>
-        <a:ln>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -3090,7 +3090,9 @@
       <c r="Q48" s="21" t="n">
         <v>1.52</v>
       </c>
-      <c r="R48" s="21" t="n"/>
+      <c r="R48" s="21" t="n">
+        <v>1.295</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="1" t="n">

</xml_diff>

<commit_message>
FIX DATOS: corrige desfase de 1 semana en serie historica de España (venia del Excel original)
- La serie España iba 1 semana tarde (mostraba el precio de la semana anterior). Verificado contra los PDF oficiales de Mercolleida (archivo de Daniel).
- Reconstruida desde el oficial: ahora coincide EXACTO (sem47/2025 = 1,314 real, no 1,354).
- Francia/Alemania estaban bien, no se tocan.
- Impacto en el modelo: MAE 0,66->0,71 cts (el desfase daba una pizca de ventaja; sigue siendo ~0,7, honesto). Pred sem41 1,268->1,270.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/master.xlsx
+++ b/data/master.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="3" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="CEBADO LLEIDA" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="ALEMANIA" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="FRANCIA" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="DINAMARCA" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CEBADO LLEIDA" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ALEMANIA" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FRANCIA" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DINAMARCA" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="145621" fullCalcOnLoad="1"/>
@@ -299,7 +299,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor editAs="oneCell">
     <from>
       <col>0</col>
@@ -317,26 +317,26 @@
       <nvPicPr>
         <cNvPr id="2" name="1 Imagen"/>
         <cNvPicPr>
-          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1" noChangeArrowheads="1"/>
         </cNvPicPr>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId1"/>
-        <a:srcRect/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:srcRect xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr bwMode="auto">
-        <a:xfrm>
+        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:off x="464691" y="60960"/>
           <a:ext cx="1646177" cy="487680"/>
         </a:xfrm>
-        <a:prstGeom prst="rect">
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
           <avLst/>
         </a:prstGeom>
-        <a:noFill/>
-        <a:ln>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -348,7 +348,7 @@
 </file>
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor editAs="oneCell">
     <from>
       <col>0</col>
@@ -366,26 +366,26 @@
       <nvPicPr>
         <cNvPr id="2" name="1 Imagen"/>
         <cNvPicPr>
-          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1" noChangeArrowheads="1"/>
         </cNvPicPr>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId1"/>
-        <a:srcRect/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:srcRect xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr bwMode="auto">
-        <a:xfrm>
+        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:off x="478979" y="60960"/>
           <a:ext cx="1646177" cy="487680"/>
         </a:xfrm>
-        <a:prstGeom prst="rect">
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
           <avLst/>
         </a:prstGeom>
-        <a:noFill/>
-        <a:ln>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -397,7 +397,7 @@
 </file>
 
 <file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor editAs="oneCell">
     <from>
       <col>0</col>
@@ -415,26 +415,26 @@
       <nvPicPr>
         <cNvPr id="2" name="1 Imagen"/>
         <cNvPicPr>
-          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1" noChangeArrowheads="1"/>
         </cNvPicPr>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId1"/>
-        <a:srcRect/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:srcRect xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr bwMode="auto">
-        <a:xfrm>
+        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:off x="478979" y="60960"/>
           <a:ext cx="1646177" cy="487680"/>
         </a:xfrm>
-        <a:prstGeom prst="rect">
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
           <avLst/>
         </a:prstGeom>
-        <a:noFill/>
-        <a:ln>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -446,7 +446,7 @@
 </file>
 
 <file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor editAs="oneCell">
     <from>
       <col>0</col>
@@ -464,26 +464,26 @@
       <nvPicPr>
         <cNvPr id="2" name="1 Imagen"/>
         <cNvPicPr>
-          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1" noChangeArrowheads="1"/>
         </cNvPicPr>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId1"/>
-        <a:srcRect/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:srcRect xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr bwMode="auto">
-        <a:xfrm>
+        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:off x="478979" y="60960"/>
           <a:ext cx="1646177" cy="487680"/>
         </a:xfrm>
-        <a:prstGeom prst="rect">
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
           <avLst/>
         </a:prstGeom>
-        <a:noFill/>
-        <a:ln>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -865,28 +865,28 @@
         <v>1.03</v>
       </c>
       <c r="D9" s="21" t="n">
-        <v>1.127</v>
+        <v>1.12</v>
       </c>
       <c r="E9" s="21" t="n">
         <v>1.303</v>
       </c>
       <c r="F9" s="21" t="n">
-        <v>1.253</v>
+        <v>1.223</v>
       </c>
       <c r="G9" s="21" t="n">
-        <v>1.043</v>
+        <v>1.033</v>
       </c>
       <c r="H9" s="21" t="n">
         <v>0.947</v>
       </c>
       <c r="I9" s="21" t="n">
-        <v>1.129</v>
+        <v>1.133</v>
       </c>
       <c r="J9" s="21" t="n">
-        <v>1.015</v>
+        <v>1.007</v>
       </c>
       <c r="K9" s="21" t="n">
-        <v>1.038</v>
+        <v>1.036</v>
       </c>
       <c r="L9" s="21" t="n">
         <v>1.49</v>
@@ -915,55 +915,55 @@
         <v>2</v>
       </c>
       <c r="B10" s="20" t="n">
-        <v>1.005</v>
+        <v>1.006</v>
       </c>
       <c r="C10" s="20" t="n">
-        <v>1.03</v>
+        <v>1.06</v>
       </c>
       <c r="D10" s="21" t="n">
-        <v>1.12</v>
+        <v>1.102</v>
       </c>
       <c r="E10" s="21" t="n">
         <v>1.303</v>
       </c>
       <c r="F10" s="21" t="n">
-        <v>1.223</v>
+        <v>1.211</v>
       </c>
       <c r="G10" s="21" t="n">
-        <v>1.033</v>
+        <v>1.023</v>
       </c>
       <c r="H10" s="21" t="n">
-        <v>0.947</v>
+        <v>0.948</v>
       </c>
       <c r="I10" s="21" t="n">
-        <v>1.133</v>
+        <v>1.132</v>
       </c>
       <c r="J10" s="21" t="n">
-        <v>1.007</v>
+        <v>0.999</v>
       </c>
       <c r="K10" s="21" t="n">
         <v>1.036</v>
       </c>
       <c r="L10" s="21" t="n">
-        <v>1.49</v>
+        <v>1.447</v>
       </c>
       <c r="M10" s="21" t="n">
         <v>1.096</v>
       </c>
       <c r="N10" s="21" t="n">
-        <v>1.02</v>
+        <v>1.021</v>
       </c>
       <c r="O10" s="21" t="n">
-        <v>1.645</v>
+        <v>1.665</v>
       </c>
       <c r="P10" s="21" t="n">
         <v>1.634</v>
       </c>
       <c r="Q10" s="21" t="n">
-        <v>1.565</v>
+        <v>1.555</v>
       </c>
       <c r="R10" s="21" t="n">
-        <v>1.04</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11">
@@ -971,10 +971,10 @@
         <v>3</v>
       </c>
       <c r="B11" s="20" t="n">
-        <v>1.006</v>
+        <v>1.015</v>
       </c>
       <c r="C11" s="20" t="n">
-        <v>1.06</v>
+        <v>1.087</v>
       </c>
       <c r="D11" s="21" t="n">
         <v>1.102</v>
@@ -986,37 +986,37 @@
         <v>1.211</v>
       </c>
       <c r="G11" s="21" t="n">
-        <v>1.023</v>
+        <v>1.018</v>
       </c>
       <c r="H11" s="21" t="n">
-        <v>0.948</v>
+        <v>0.951</v>
       </c>
       <c r="I11" s="21" t="n">
         <v>1.132</v>
       </c>
       <c r="J11" s="21" t="n">
-        <v>0.999</v>
+        <v>0.995</v>
       </c>
       <c r="K11" s="21" t="n">
         <v>1.036</v>
       </c>
       <c r="L11" s="21" t="n">
-        <v>1.447</v>
+        <v>1.42</v>
       </c>
       <c r="M11" s="21" t="n">
         <v>1.096</v>
       </c>
       <c r="N11" s="21" t="n">
-        <v>1.021</v>
+        <v>1.022</v>
       </c>
       <c r="O11" s="21" t="n">
-        <v>1.665</v>
+        <v>1.69</v>
       </c>
       <c r="P11" s="21" t="n">
         <v>1.634</v>
       </c>
       <c r="Q11" s="21" t="n">
-        <v>1.555</v>
+        <v>1.54</v>
       </c>
       <c r="R11" s="21" t="n">
         <v>1</v>
@@ -1027,28 +1027,28 @@
         <v>4</v>
       </c>
       <c r="B12" s="20" t="n">
-        <v>1.015</v>
+        <v>1.032</v>
       </c>
       <c r="C12" s="20" t="n">
-        <v>1.087</v>
+        <v>1.125</v>
       </c>
       <c r="D12" s="21" t="n">
-        <v>1.102</v>
+        <v>1.127</v>
       </c>
       <c r="E12" s="21" t="n">
         <v>1.303</v>
       </c>
       <c r="F12" s="21" t="n">
-        <v>1.211</v>
+        <v>1.215</v>
       </c>
       <c r="G12" s="21" t="n">
-        <v>1.018</v>
+        <v>1.02</v>
       </c>
       <c r="H12" s="21" t="n">
-        <v>0.951</v>
+        <v>0.956</v>
       </c>
       <c r="I12" s="21" t="n">
-        <v>1.132</v>
+        <v>1.149</v>
       </c>
       <c r="J12" s="21" t="n">
         <v>0.995</v>
@@ -1060,13 +1060,13 @@
         <v>1.42</v>
       </c>
       <c r="M12" s="21" t="n">
-        <v>1.096</v>
+        <v>1.1</v>
       </c>
       <c r="N12" s="21" t="n">
-        <v>1.022</v>
+        <v>1.035</v>
       </c>
       <c r="O12" s="21" t="n">
-        <v>1.69</v>
+        <v>1.718</v>
       </c>
       <c r="P12" s="21" t="n">
         <v>1.634</v>
@@ -1083,46 +1083,46 @@
         <v>5</v>
       </c>
       <c r="B13" s="20" t="n">
-        <v>1.032</v>
+        <v>1.06</v>
       </c>
       <c r="C13" s="20" t="n">
-        <v>1.125</v>
+        <v>1.17</v>
       </c>
       <c r="D13" s="21" t="n">
-        <v>1.127</v>
+        <v>1.161</v>
       </c>
       <c r="E13" s="21" t="n">
-        <v>1.303</v>
+        <v>1.317</v>
       </c>
       <c r="F13" s="21" t="n">
-        <v>1.215</v>
+        <v>1.227</v>
       </c>
       <c r="G13" s="21" t="n">
-        <v>1.02</v>
+        <v>1.03</v>
       </c>
       <c r="H13" s="21" t="n">
-        <v>0.956</v>
+        <v>0.967</v>
       </c>
       <c r="I13" s="21" t="n">
-        <v>1.149</v>
+        <v>1.156</v>
       </c>
       <c r="J13" s="21" t="n">
-        <v>0.995</v>
+        <v>1.005</v>
       </c>
       <c r="K13" s="21" t="n">
-        <v>1.036</v>
+        <v>1.04</v>
       </c>
       <c r="L13" s="21" t="n">
-        <v>1.42</v>
+        <v>1.424</v>
       </c>
       <c r="M13" s="21" t="n">
-        <v>1.1</v>
+        <v>1.117</v>
       </c>
       <c r="N13" s="21" t="n">
-        <v>1.035</v>
+        <v>1.059</v>
       </c>
       <c r="O13" s="21" t="n">
-        <v>1.718</v>
+        <v>1.75</v>
       </c>
       <c r="P13" s="21" t="n">
         <v>1.634</v>
@@ -1139,52 +1139,52 @@
         <v>6</v>
       </c>
       <c r="B14" s="20" t="n">
-        <v>1.06</v>
+        <v>1.1</v>
       </c>
       <c r="C14" s="20" t="n">
-        <v>1.17</v>
+        <v>1.213</v>
       </c>
       <c r="D14" s="21" t="n">
-        <v>1.161</v>
+        <v>1.2</v>
       </c>
       <c r="E14" s="21" t="n">
-        <v>1.317</v>
+        <v>1.334</v>
       </c>
       <c r="F14" s="21" t="n">
-        <v>1.227</v>
+        <v>1.226</v>
       </c>
       <c r="G14" s="21" t="n">
-        <v>1.03</v>
+        <v>1.049</v>
       </c>
       <c r="H14" s="21" t="n">
-        <v>0.967</v>
+        <v>0.971</v>
       </c>
       <c r="I14" s="21" t="n">
-        <v>1.156</v>
+        <v>1.169</v>
       </c>
       <c r="J14" s="21" t="n">
-        <v>1.005</v>
+        <v>1.035</v>
       </c>
       <c r="K14" s="21" t="n">
-        <v>1.04</v>
+        <v>1.065</v>
       </c>
       <c r="L14" s="21" t="n">
-        <v>1.424</v>
+        <v>1.427</v>
       </c>
       <c r="M14" s="21" t="n">
-        <v>1.117</v>
+        <v>1.141</v>
       </c>
       <c r="N14" s="21" t="n">
-        <v>1.059</v>
+        <v>1.088</v>
       </c>
       <c r="O14" s="21" t="n">
-        <v>1.75</v>
+        <v>1.795</v>
       </c>
       <c r="P14" s="21" t="n">
-        <v>1.634</v>
+        <v>1.651</v>
       </c>
       <c r="Q14" s="21" t="n">
-        <v>1.54</v>
+        <v>1.552</v>
       </c>
       <c r="R14" s="21" t="n">
         <v>1</v>
@@ -1195,55 +1195,55 @@
         <v>7</v>
       </c>
       <c r="B15" s="20" t="n">
-        <v>1.1</v>
+        <v>1.13</v>
       </c>
       <c r="C15" s="20" t="n">
-        <v>1.213</v>
+        <v>1.243</v>
       </c>
       <c r="D15" s="21" t="n">
+        <v>1.244</v>
+      </c>
+      <c r="E15" s="21" t="n">
+        <v>1.358</v>
+      </c>
+      <c r="F15" s="21" t="n">
         <v>1.2</v>
       </c>
-      <c r="E15" s="21" t="n">
-        <v>1.334</v>
-      </c>
-      <c r="F15" s="21" t="n">
-        <v>1.226</v>
-      </c>
       <c r="G15" s="21" t="n">
-        <v>1.049</v>
+        <v>1.08</v>
       </c>
       <c r="H15" s="21" t="n">
-        <v>0.971</v>
+        <v>0.96</v>
       </c>
       <c r="I15" s="21" t="n">
-        <v>1.169</v>
+        <v>1.182</v>
       </c>
       <c r="J15" s="21" t="n">
-        <v>1.035</v>
+        <v>1.076</v>
       </c>
       <c r="K15" s="21" t="n">
-        <v>1.065</v>
+        <v>1.09</v>
       </c>
       <c r="L15" s="21" t="n">
-        <v>1.427</v>
+        <v>1.457</v>
       </c>
       <c r="M15" s="21" t="n">
-        <v>1.141</v>
+        <v>1.178</v>
       </c>
       <c r="N15" s="21" t="n">
-        <v>1.088</v>
+        <v>1.125</v>
       </c>
       <c r="O15" s="21" t="n">
-        <v>1.795</v>
+        <v>1.845</v>
       </c>
       <c r="P15" s="21" t="n">
-        <v>1.651</v>
+        <v>1.681</v>
       </c>
       <c r="Q15" s="21" t="n">
-        <v>1.552</v>
+        <v>1.572</v>
       </c>
       <c r="R15" s="21" t="n">
-        <v>1</v>
+        <v>1.015</v>
       </c>
     </row>
     <row r="16">
@@ -1251,55 +1251,55 @@
         <v>8</v>
       </c>
       <c r="B16" s="20" t="n">
-        <v>1.13</v>
+        <v>1.145</v>
       </c>
       <c r="C16" s="20" t="n">
-        <v>1.243</v>
+        <v>1.26</v>
       </c>
       <c r="D16" s="21" t="n">
-        <v>1.244</v>
+        <v>1.284</v>
       </c>
       <c r="E16" s="21" t="n">
-        <v>1.358</v>
+        <v>1.37</v>
       </c>
       <c r="F16" s="21" t="n">
-        <v>1.2</v>
+        <v>1.198</v>
       </c>
       <c r="G16" s="21" t="n">
-        <v>1.08</v>
+        <v>1.125</v>
       </c>
       <c r="H16" s="21" t="n">
-        <v>0.96</v>
+        <v>0.9389999999999999</v>
       </c>
       <c r="I16" s="21" t="n">
-        <v>1.182</v>
+        <v>1.198</v>
       </c>
       <c r="J16" s="21" t="n">
-        <v>1.076</v>
+        <v>1.115</v>
       </c>
       <c r="K16" s="21" t="n">
-        <v>1.09</v>
+        <v>1.112</v>
       </c>
       <c r="L16" s="21" t="n">
-        <v>1.457</v>
+        <v>1.487</v>
       </c>
       <c r="M16" s="21" t="n">
-        <v>1.178</v>
+        <v>1.235</v>
       </c>
       <c r="N16" s="21" t="n">
-        <v>1.125</v>
+        <v>1.172</v>
       </c>
       <c r="O16" s="21" t="n">
-        <v>1.845</v>
+        <v>1.89</v>
       </c>
       <c r="P16" s="21" t="n">
-        <v>1.681</v>
+        <v>1.708</v>
       </c>
       <c r="Q16" s="21" t="n">
-        <v>1.572</v>
+        <v>1.597</v>
       </c>
       <c r="R16" s="21" t="n">
-        <v>1.015</v>
+        <v>1.05</v>
       </c>
     </row>
     <row r="17">
@@ -1307,55 +1307,55 @@
         <v>9</v>
       </c>
       <c r="B17" s="20" t="n">
+        <v>1.137</v>
+      </c>
+      <c r="C17" s="20" t="n">
+        <v>1.265</v>
+      </c>
+      <c r="D17" s="21" t="n">
+        <v>1.294</v>
+      </c>
+      <c r="E17" s="21" t="n">
+        <v>1.374</v>
+      </c>
+      <c r="F17" s="21" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="G17" s="21" t="n">
         <v>1.145</v>
-      </c>
-      <c r="C17" s="20" t="n">
-        <v>1.26</v>
-      </c>
-      <c r="D17" s="21" t="n">
-        <v>1.284</v>
-      </c>
-      <c r="E17" s="21" t="n">
-        <v>1.37</v>
-      </c>
-      <c r="F17" s="21" t="n">
-        <v>1.198</v>
-      </c>
-      <c r="G17" s="21" t="n">
-        <v>1.125</v>
       </c>
       <c r="H17" s="21" t="n">
         <v>0.9389999999999999</v>
       </c>
       <c r="I17" s="21" t="n">
-        <v>1.198</v>
+        <v>1.218</v>
       </c>
       <c r="J17" s="21" t="n">
-        <v>1.115</v>
+        <v>1.146</v>
       </c>
       <c r="K17" s="21" t="n">
-        <v>1.112</v>
+        <v>1.133</v>
       </c>
       <c r="L17" s="21" t="n">
-        <v>1.487</v>
+        <v>1.522</v>
       </c>
       <c r="M17" s="21" t="n">
-        <v>1.235</v>
+        <v>1.295</v>
       </c>
       <c r="N17" s="21" t="n">
-        <v>1.172</v>
+        <v>1.232</v>
       </c>
       <c r="O17" s="21" t="n">
-        <v>1.89</v>
+        <v>1.932</v>
       </c>
       <c r="P17" s="21" t="n">
-        <v>1.708</v>
+        <v>1.738</v>
       </c>
       <c r="Q17" s="21" t="n">
-        <v>1.597</v>
+        <v>1.627</v>
       </c>
       <c r="R17" s="21" t="n">
-        <v>1.05</v>
+        <v>1.095</v>
       </c>
     </row>
     <row r="18">
@@ -1363,7 +1363,7 @@
         <v>10</v>
       </c>
       <c r="B18" s="20" t="n">
-        <v>1.137</v>
+        <v>1.117</v>
       </c>
       <c r="C18" s="20" t="n">
         <v>1.265</v>
@@ -1372,46 +1372,46 @@
         <v>1.294</v>
       </c>
       <c r="E18" s="21" t="n">
-        <v>1.374</v>
+        <v>1.377</v>
       </c>
       <c r="F18" s="21" t="n">
         <v>1.2</v>
       </c>
       <c r="G18" s="21" t="n">
+        <v>1.148</v>
+      </c>
+      <c r="H18" s="21" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="I18" s="21" t="n">
+        <v>1.24</v>
+      </c>
+      <c r="J18" s="21" t="n">
+        <v>1.156</v>
+      </c>
+      <c r="K18" s="21" t="n">
+        <v>1.155</v>
+      </c>
+      <c r="L18" s="21" t="n">
+        <v>1.54</v>
+      </c>
+      <c r="M18" s="21" t="n">
+        <v>1.355</v>
+      </c>
+      <c r="N18" s="21" t="n">
+        <v>1.292</v>
+      </c>
+      <c r="O18" s="21" t="n">
+        <v>1.967</v>
+      </c>
+      <c r="P18" s="21" t="n">
+        <v>1.766</v>
+      </c>
+      <c r="Q18" s="21" t="n">
+        <v>1.657</v>
+      </c>
+      <c r="R18" s="21" t="n">
         <v>1.145</v>
-      </c>
-      <c r="H18" s="21" t="n">
-        <v>0.9389999999999999</v>
-      </c>
-      <c r="I18" s="21" t="n">
-        <v>1.218</v>
-      </c>
-      <c r="J18" s="21" t="n">
-        <v>1.146</v>
-      </c>
-      <c r="K18" s="21" t="n">
-        <v>1.133</v>
-      </c>
-      <c r="L18" s="21" t="n">
-        <v>1.522</v>
-      </c>
-      <c r="M18" s="21" t="n">
-        <v>1.295</v>
-      </c>
-      <c r="N18" s="21" t="n">
-        <v>1.232</v>
-      </c>
-      <c r="O18" s="21" t="n">
-        <v>1.932</v>
-      </c>
-      <c r="P18" s="21" t="n">
-        <v>1.738</v>
-      </c>
-      <c r="Q18" s="21" t="n">
-        <v>1.627</v>
-      </c>
-      <c r="R18" s="21" t="n">
-        <v>1.095</v>
       </c>
     </row>
     <row r="19">
@@ -1419,7 +1419,7 @@
         <v>11</v>
       </c>
       <c r="B19" s="20" t="n">
-        <v>1.117</v>
+        <v>1.07</v>
       </c>
       <c r="C19" s="20" t="n">
         <v>1.265</v>
@@ -1437,37 +1437,37 @@
         <v>1.148</v>
       </c>
       <c r="H19" s="21" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.955</v>
       </c>
       <c r="I19" s="21" t="n">
-        <v>1.24</v>
+        <v>1.25</v>
       </c>
       <c r="J19" s="21" t="n">
         <v>1.156</v>
       </c>
       <c r="K19" s="21" t="n">
-        <v>1.155</v>
+        <v>1.184</v>
       </c>
       <c r="L19" s="21" t="n">
         <v>1.54</v>
       </c>
       <c r="M19" s="21" t="n">
-        <v>1.355</v>
+        <v>1.41</v>
       </c>
       <c r="N19" s="21" t="n">
-        <v>1.292</v>
+        <v>1.352</v>
       </c>
       <c r="O19" s="21" t="n">
-        <v>1.967</v>
+        <v>1.995</v>
       </c>
       <c r="P19" s="21" t="n">
-        <v>1.766</v>
+        <v>1.788</v>
       </c>
       <c r="Q19" s="21" t="n">
-        <v>1.657</v>
+        <v>1.685</v>
       </c>
       <c r="R19" s="21" t="n">
-        <v>1.145</v>
+        <v>1.205</v>
       </c>
     </row>
     <row r="20">
@@ -1475,7 +1475,7 @@
         <v>12</v>
       </c>
       <c r="B20" s="20" t="n">
-        <v>1.07</v>
+        <v>1.042</v>
       </c>
       <c r="C20" s="20" t="n">
         <v>1.265</v>
@@ -1487,7 +1487,7 @@
         <v>1.377</v>
       </c>
       <c r="F20" s="21" t="n">
-        <v>1.2</v>
+        <v>1.25</v>
       </c>
       <c r="G20" s="21" t="n">
         <v>1.148</v>
@@ -1496,34 +1496,34 @@
         <v>0.955</v>
       </c>
       <c r="I20" s="21" t="n">
-        <v>1.25</v>
+        <v>1.275</v>
       </c>
       <c r="J20" s="21" t="n">
         <v>1.156</v>
       </c>
       <c r="K20" s="21" t="n">
-        <v>1.184</v>
+        <v>1.223</v>
       </c>
       <c r="L20" s="21" t="n">
-        <v>1.54</v>
+        <v>1.51</v>
       </c>
       <c r="M20" s="21" t="n">
-        <v>1.41</v>
+        <v>1.46</v>
       </c>
       <c r="N20" s="21" t="n">
-        <v>1.352</v>
+        <v>1.412</v>
       </c>
       <c r="O20" s="21" t="n">
-        <v>1.995</v>
+        <v>2.015</v>
       </c>
       <c r="P20" s="21" t="n">
-        <v>1.788</v>
+        <v>1.8</v>
       </c>
       <c r="Q20" s="21" t="n">
-        <v>1.685</v>
+        <v>1.706</v>
       </c>
       <c r="R20" s="21" t="n">
-        <v>1.205</v>
+        <v>1.245</v>
       </c>
     </row>
     <row r="21">
@@ -1531,7 +1531,7 @@
         <v>13</v>
       </c>
       <c r="B21" s="20" t="n">
-        <v>1.042</v>
+        <v>1.03</v>
       </c>
       <c r="C21" s="20" t="n">
         <v>1.265</v>
@@ -1543,43 +1543,43 @@
         <v>1.377</v>
       </c>
       <c r="F21" s="21" t="n">
-        <v>1.25</v>
+        <v>1.275</v>
       </c>
       <c r="G21" s="21" t="n">
         <v>1.148</v>
       </c>
       <c r="H21" s="21" t="n">
-        <v>0.955</v>
+        <v>0.95</v>
       </c>
       <c r="I21" s="21" t="n">
-        <v>1.275</v>
+        <v>1.31</v>
       </c>
       <c r="J21" s="21" t="n">
         <v>1.156</v>
       </c>
       <c r="K21" s="21" t="n">
-        <v>1.223</v>
+        <v>1.274</v>
       </c>
       <c r="L21" s="21" t="n">
-        <v>1.51</v>
+        <v>1.49</v>
       </c>
       <c r="M21" s="21" t="n">
         <v>1.46</v>
       </c>
       <c r="N21" s="21" t="n">
-        <v>1.412</v>
+        <v>1.472</v>
       </c>
       <c r="O21" s="21" t="n">
-        <v>2.015</v>
+        <v>2.025</v>
       </c>
       <c r="P21" s="21" t="n">
         <v>1.8</v>
       </c>
       <c r="Q21" s="21" t="n">
-        <v>1.706</v>
+        <v>1.727</v>
       </c>
       <c r="R21" s="21" t="n">
-        <v>1.245</v>
+        <v>1.27</v>
       </c>
     </row>
     <row r="22">
@@ -1599,7 +1599,7 @@
         <v>1.377</v>
       </c>
       <c r="F22" s="21" t="n">
-        <v>1.275</v>
+        <v>1.315</v>
       </c>
       <c r="G22" s="21" t="n">
         <v>1.148</v>
@@ -1608,22 +1608,22 @@
         <v>0.95</v>
       </c>
       <c r="I22" s="21" t="n">
-        <v>1.31</v>
+        <v>1.355</v>
       </c>
       <c r="J22" s="21" t="n">
         <v>1.156</v>
       </c>
       <c r="K22" s="21" t="n">
-        <v>1.274</v>
+        <v>1.33</v>
       </c>
       <c r="L22" s="21" t="n">
-        <v>1.49</v>
+        <v>1.475</v>
       </c>
       <c r="M22" s="21" t="n">
         <v>1.46</v>
       </c>
       <c r="N22" s="21" t="n">
-        <v>1.472</v>
+        <v>1.53</v>
       </c>
       <c r="O22" s="21" t="n">
         <v>2.025</v>
@@ -1632,7 +1632,7 @@
         <v>1.8</v>
       </c>
       <c r="Q22" s="21" t="n">
-        <v>1.727</v>
+        <v>1.748</v>
       </c>
       <c r="R22" s="21" t="n">
         <v>1.27</v>
@@ -1655,13 +1655,13 @@
         <v>1.377</v>
       </c>
       <c r="F23" s="21" t="n">
-        <v>1.315</v>
+        <v>1.36</v>
       </c>
       <c r="G23" s="21" t="n">
-        <v>1.148</v>
+        <v>1.154</v>
       </c>
       <c r="H23" s="21" t="n">
-        <v>0.95</v>
+        <v>0.952</v>
       </c>
       <c r="I23" s="21" t="n">
         <v>1.355</v>
@@ -1670,10 +1670,10 @@
         <v>1.156</v>
       </c>
       <c r="K23" s="21" t="n">
-        <v>1.33</v>
+        <v>1.36</v>
       </c>
       <c r="L23" s="21" t="n">
-        <v>1.475</v>
+        <v>1.455</v>
       </c>
       <c r="M23" s="21" t="n">
         <v>1.46</v>
@@ -1688,7 +1688,7 @@
         <v>1.8</v>
       </c>
       <c r="Q23" s="21" t="n">
-        <v>1.748</v>
+        <v>1.774</v>
       </c>
       <c r="R23" s="21" t="n">
         <v>1.27</v>
@@ -1699,7 +1699,7 @@
         <v>16</v>
       </c>
       <c r="B24" s="20" t="n">
-        <v>1.03</v>
+        <v>1.05</v>
       </c>
       <c r="C24" s="20" t="n">
         <v>1.265</v>
@@ -1714,10 +1714,10 @@
         <v>1.36</v>
       </c>
       <c r="G24" s="21" t="n">
-        <v>1.154</v>
+        <v>1.177</v>
       </c>
       <c r="H24" s="21" t="n">
-        <v>0.952</v>
+        <v>0.96</v>
       </c>
       <c r="I24" s="21" t="n">
         <v>1.355</v>
@@ -1729,13 +1729,13 @@
         <v>1.36</v>
       </c>
       <c r="L24" s="21" t="n">
-        <v>1.455</v>
+        <v>1.433</v>
       </c>
       <c r="M24" s="21" t="n">
         <v>1.46</v>
       </c>
       <c r="N24" s="21" t="n">
-        <v>1.53</v>
+        <v>1.54</v>
       </c>
       <c r="O24" s="21" t="n">
         <v>2.025</v>
@@ -1755,25 +1755,25 @@
         <v>17</v>
       </c>
       <c r="B25" s="20" t="n">
-        <v>1.05</v>
+        <v>1.087</v>
       </c>
       <c r="C25" s="20" t="n">
-        <v>1.265</v>
+        <v>1.282</v>
       </c>
       <c r="D25" s="21" t="n">
         <v>1.294</v>
       </c>
       <c r="E25" s="21" t="n">
-        <v>1.377</v>
+        <v>1.37</v>
       </c>
       <c r="F25" s="21" t="n">
         <v>1.36</v>
       </c>
       <c r="G25" s="21" t="n">
-        <v>1.177</v>
+        <v>1.185</v>
       </c>
       <c r="H25" s="21" t="n">
-        <v>0.96</v>
+        <v>0.985</v>
       </c>
       <c r="I25" s="21" t="n">
         <v>1.355</v>
@@ -1785,13 +1785,13 @@
         <v>1.36</v>
       </c>
       <c r="L25" s="21" t="n">
-        <v>1.433</v>
+        <v>1.388</v>
       </c>
       <c r="M25" s="21" t="n">
         <v>1.46</v>
       </c>
       <c r="N25" s="21" t="n">
-        <v>1.54</v>
+        <v>1.545</v>
       </c>
       <c r="O25" s="21" t="n">
         <v>2.025</v>
@@ -1811,25 +1811,25 @@
         <v>18</v>
       </c>
       <c r="B26" s="20" t="n">
-        <v>1.087</v>
+        <v>1.124</v>
       </c>
       <c r="C26" s="20" t="n">
-        <v>1.282</v>
+        <v>1.295</v>
       </c>
       <c r="D26" s="21" t="n">
         <v>1.294</v>
       </c>
       <c r="E26" s="21" t="n">
-        <v>1.37</v>
+        <v>1.343</v>
       </c>
       <c r="F26" s="21" t="n">
-        <v>1.36</v>
+        <v>1.365</v>
       </c>
       <c r="G26" s="21" t="n">
-        <v>1.185</v>
+        <v>1.178</v>
       </c>
       <c r="H26" s="21" t="n">
-        <v>0.985</v>
+        <v>1.027</v>
       </c>
       <c r="I26" s="21" t="n">
         <v>1.355</v>
@@ -1841,10 +1841,10 @@
         <v>1.36</v>
       </c>
       <c r="L26" s="21" t="n">
-        <v>1.388</v>
+        <v>1.343</v>
       </c>
       <c r="M26" s="21" t="n">
-        <v>1.46</v>
+        <v>1.47</v>
       </c>
       <c r="N26" s="21" t="n">
         <v>1.545</v>
@@ -1867,7 +1867,7 @@
         <v>19</v>
       </c>
       <c r="B27" s="20" t="n">
-        <v>1.124</v>
+        <v>1.148</v>
       </c>
       <c r="C27" s="20" t="n">
         <v>1.295</v>
@@ -1876,16 +1876,16 @@
         <v>1.294</v>
       </c>
       <c r="E27" s="21" t="n">
-        <v>1.343</v>
+        <v>1.326</v>
       </c>
       <c r="F27" s="21" t="n">
         <v>1.365</v>
       </c>
       <c r="G27" s="21" t="n">
-        <v>1.178</v>
+        <v>1.174</v>
       </c>
       <c r="H27" s="21" t="n">
-        <v>1.027</v>
+        <v>1.07</v>
       </c>
       <c r="I27" s="21" t="n">
         <v>1.355</v>
@@ -1894,13 +1894,13 @@
         <v>1.156</v>
       </c>
       <c r="K27" s="21" t="n">
-        <v>1.36</v>
+        <v>1.371</v>
       </c>
       <c r="L27" s="21" t="n">
-        <v>1.343</v>
+        <v>1.29</v>
       </c>
       <c r="M27" s="21" t="n">
-        <v>1.47</v>
+        <v>1.49</v>
       </c>
       <c r="N27" s="21" t="n">
         <v>1.545</v>
@@ -1923,40 +1923,40 @@
         <v>20</v>
       </c>
       <c r="B28" s="20" t="n">
-        <v>1.148</v>
+        <v>1.18</v>
       </c>
       <c r="C28" s="20" t="n">
-        <v>1.295</v>
+        <v>1.28</v>
       </c>
       <c r="D28" s="21" t="n">
-        <v>1.294</v>
+        <v>1.31</v>
       </c>
       <c r="E28" s="21" t="n">
         <v>1.326</v>
       </c>
       <c r="F28" s="21" t="n">
-        <v>1.365</v>
+        <v>1.361</v>
       </c>
       <c r="G28" s="21" t="n">
         <v>1.174</v>
       </c>
       <c r="H28" s="21" t="n">
-        <v>1.07</v>
+        <v>1.097</v>
       </c>
       <c r="I28" s="21" t="n">
-        <v>1.355</v>
+        <v>1.365</v>
       </c>
       <c r="J28" s="21" t="n">
-        <v>1.156</v>
+        <v>1.164</v>
       </c>
       <c r="K28" s="21" t="n">
-        <v>1.371</v>
+        <v>1.392</v>
       </c>
       <c r="L28" s="21" t="n">
-        <v>1.29</v>
+        <v>1.263</v>
       </c>
       <c r="M28" s="21" t="n">
-        <v>1.49</v>
+        <v>1.518</v>
       </c>
       <c r="N28" s="21" t="n">
         <v>1.545</v>
@@ -1979,43 +1979,43 @@
         <v>21</v>
       </c>
       <c r="B29" s="20" t="n">
-        <v>1.18</v>
+        <v>1.205</v>
       </c>
       <c r="C29" s="20" t="n">
-        <v>1.28</v>
+        <v>1.26</v>
       </c>
       <c r="D29" s="21" t="n">
-        <v>1.31</v>
+        <v>1.337</v>
       </c>
       <c r="E29" s="21" t="n">
         <v>1.326</v>
       </c>
       <c r="F29" s="21" t="n">
-        <v>1.361</v>
+        <v>1.378</v>
       </c>
       <c r="G29" s="21" t="n">
-        <v>1.174</v>
+        <v>1.185</v>
       </c>
       <c r="H29" s="21" t="n">
-        <v>1.097</v>
+        <v>1.143</v>
       </c>
       <c r="I29" s="21" t="n">
-        <v>1.365</v>
+        <v>1.375</v>
       </c>
       <c r="J29" s="21" t="n">
-        <v>1.164</v>
+        <v>1.18</v>
       </c>
       <c r="K29" s="21" t="n">
-        <v>1.392</v>
+        <v>1.408</v>
       </c>
       <c r="L29" s="21" t="n">
-        <v>1.263</v>
+        <v>1.264</v>
       </c>
       <c r="M29" s="21" t="n">
-        <v>1.518</v>
+        <v>1.535</v>
       </c>
       <c r="N29" s="21" t="n">
-        <v>1.545</v>
+        <v>1.549</v>
       </c>
       <c r="O29" s="21" t="n">
         <v>2.025</v>
@@ -2024,10 +2024,10 @@
         <v>1.8</v>
       </c>
       <c r="Q29" s="21" t="n">
-        <v>1.774</v>
+        <v>1.779</v>
       </c>
       <c r="R29" s="21" t="n">
-        <v>1.27</v>
+        <v>1.275</v>
       </c>
     </row>
     <row r="30">
@@ -2035,43 +2035,43 @@
         <v>22</v>
       </c>
       <c r="B30" s="20" t="n">
-        <v>1.205</v>
+        <v>1.238</v>
       </c>
       <c r="C30" s="20" t="n">
         <v>1.26</v>
       </c>
       <c r="D30" s="21" t="n">
-        <v>1.337</v>
+        <v>1.366</v>
       </c>
       <c r="E30" s="21" t="n">
-        <v>1.326</v>
+        <v>1.33</v>
       </c>
       <c r="F30" s="21" t="n">
-        <v>1.378</v>
+        <v>1.39</v>
       </c>
       <c r="G30" s="21" t="n">
+        <v>1.198</v>
+      </c>
+      <c r="H30" s="21" t="n">
         <v>1.185</v>
       </c>
-      <c r="H30" s="21" t="n">
-        <v>1.143</v>
-      </c>
       <c r="I30" s="21" t="n">
-        <v>1.375</v>
+        <v>1.392</v>
       </c>
       <c r="J30" s="21" t="n">
-        <v>1.18</v>
+        <v>1.194</v>
       </c>
       <c r="K30" s="21" t="n">
-        <v>1.408</v>
+        <v>1.419</v>
       </c>
       <c r="L30" s="21" t="n">
-        <v>1.264</v>
+        <v>1.276</v>
       </c>
       <c r="M30" s="21" t="n">
-        <v>1.535</v>
+        <v>1.55</v>
       </c>
       <c r="N30" s="21" t="n">
-        <v>1.549</v>
+        <v>1.563</v>
       </c>
       <c r="O30" s="21" t="n">
         <v>2.025</v>
@@ -2080,10 +2080,10 @@
         <v>1.8</v>
       </c>
       <c r="Q30" s="21" t="n">
-        <v>1.779</v>
+        <v>1.787</v>
       </c>
       <c r="R30" s="21" t="n">
-        <v>1.275</v>
+        <v>1.29</v>
       </c>
     </row>
     <row r="31">
@@ -2091,55 +2091,55 @@
         <v>23</v>
       </c>
       <c r="B31" s="20" t="n">
-        <v>1.238</v>
+        <v>1.258</v>
       </c>
       <c r="C31" s="20" t="n">
-        <v>1.26</v>
+        <v>1.27</v>
       </c>
       <c r="D31" s="21" t="n">
-        <v>1.366</v>
+        <v>1.38</v>
       </c>
       <c r="E31" s="21" t="n">
-        <v>1.33</v>
+        <v>1.356</v>
       </c>
       <c r="F31" s="21" t="n">
-        <v>1.39</v>
+        <v>1.412</v>
       </c>
       <c r="G31" s="21" t="n">
-        <v>1.198</v>
+        <v>1.22</v>
       </c>
       <c r="H31" s="21" t="n">
-        <v>1.185</v>
+        <v>1.208</v>
       </c>
       <c r="I31" s="21" t="n">
-        <v>1.392</v>
+        <v>1.4</v>
       </c>
       <c r="J31" s="21" t="n">
-        <v>1.194</v>
+        <v>1.212</v>
       </c>
       <c r="K31" s="21" t="n">
-        <v>1.419</v>
+        <v>1.449</v>
       </c>
       <c r="L31" s="21" t="n">
-        <v>1.276</v>
+        <v>1.288</v>
       </c>
       <c r="M31" s="21" t="n">
-        <v>1.55</v>
+        <v>1.553</v>
       </c>
       <c r="N31" s="21" t="n">
-        <v>1.563</v>
+        <v>1.58</v>
       </c>
       <c r="O31" s="21" t="n">
         <v>2.025</v>
       </c>
       <c r="P31" s="21" t="n">
-        <v>1.8</v>
+        <v>1.805</v>
       </c>
       <c r="Q31" s="21" t="n">
-        <v>1.787</v>
+        <v>1.797</v>
       </c>
       <c r="R31" s="21" t="n">
-        <v>1.29</v>
+        <v>1.31</v>
       </c>
     </row>
     <row r="32">
@@ -2147,7 +2147,7 @@
         <v>24</v>
       </c>
       <c r="B32" s="20" t="n">
-        <v>1.258</v>
+        <v>1.271</v>
       </c>
       <c r="C32" s="20" t="n">
         <v>1.27</v>
@@ -2156,43 +2156,43 @@
         <v>1.38</v>
       </c>
       <c r="E32" s="21" t="n">
-        <v>1.356</v>
+        <v>1.396</v>
       </c>
       <c r="F32" s="21" t="n">
+        <v>1.435</v>
+      </c>
+      <c r="G32" s="21" t="n">
+        <v>1.251</v>
+      </c>
+      <c r="H32" s="21" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="I32" s="21" t="n">
         <v>1.412</v>
       </c>
-      <c r="G32" s="21" t="n">
-        <v>1.22</v>
-      </c>
-      <c r="H32" s="21" t="n">
-        <v>1.208</v>
-      </c>
-      <c r="I32" s="21" t="n">
-        <v>1.4</v>
-      </c>
       <c r="J32" s="21" t="n">
-        <v>1.212</v>
+        <v>1.215</v>
       </c>
       <c r="K32" s="21" t="n">
         <v>1.449</v>
       </c>
       <c r="L32" s="21" t="n">
-        <v>1.288</v>
+        <v>1.303</v>
       </c>
       <c r="M32" s="21" t="n">
-        <v>1.553</v>
+        <v>1.543</v>
       </c>
       <c r="N32" s="21" t="n">
-        <v>1.58</v>
+        <v>1.598</v>
       </c>
       <c r="O32" s="21" t="n">
         <v>2.025</v>
       </c>
       <c r="P32" s="21" t="n">
-        <v>1.805</v>
+        <v>1.818</v>
       </c>
       <c r="Q32" s="21" t="n">
-        <v>1.797</v>
+        <v>1.81</v>
       </c>
       <c r="R32" s="21" t="n">
         <v>1.31</v>
@@ -2212,43 +2212,43 @@
         <v>1.38</v>
       </c>
       <c r="E33" s="21" t="n">
-        <v>1.396</v>
+        <v>1.42</v>
       </c>
       <c r="F33" s="21" t="n">
-        <v>1.435</v>
+        <v>1.455</v>
       </c>
       <c r="G33" s="21" t="n">
-        <v>1.251</v>
+        <v>1.259</v>
       </c>
       <c r="H33" s="21" t="n">
-        <v>1.25</v>
+        <v>1.28</v>
       </c>
       <c r="I33" s="21" t="n">
-        <v>1.412</v>
+        <v>1.425</v>
       </c>
       <c r="J33" s="21" t="n">
-        <v>1.215</v>
+        <v>1.22</v>
       </c>
       <c r="K33" s="21" t="n">
-        <v>1.449</v>
+        <v>1.451</v>
       </c>
       <c r="L33" s="21" t="n">
-        <v>1.303</v>
+        <v>1.318</v>
       </c>
       <c r="M33" s="21" t="n">
-        <v>1.543</v>
+        <v>1.51</v>
       </c>
       <c r="N33" s="21" t="n">
-        <v>1.598</v>
+        <v>1.626</v>
       </c>
       <c r="O33" s="21" t="n">
         <v>2.025</v>
       </c>
       <c r="P33" s="21" t="n">
-        <v>1.818</v>
+        <v>1.833</v>
       </c>
       <c r="Q33" s="21" t="n">
-        <v>1.81</v>
+        <v>1.815</v>
       </c>
       <c r="R33" s="21" t="n">
         <v>1.31</v>
@@ -2268,40 +2268,40 @@
         <v>1.38</v>
       </c>
       <c r="E34" s="21" t="n">
-        <v>1.42</v>
+        <v>1.43</v>
       </c>
       <c r="F34" s="21" t="n">
-        <v>1.455</v>
+        <v>1.475</v>
       </c>
       <c r="G34" s="21" t="n">
-        <v>1.259</v>
+        <v>1.256</v>
       </c>
       <c r="H34" s="21" t="n">
-        <v>1.28</v>
+        <v>1.3</v>
       </c>
       <c r="I34" s="21" t="n">
-        <v>1.425</v>
+        <v>1.435</v>
       </c>
       <c r="J34" s="21" t="n">
-        <v>1.22</v>
+        <v>1.23</v>
       </c>
       <c r="K34" s="21" t="n">
         <v>1.451</v>
       </c>
       <c r="L34" s="21" t="n">
-        <v>1.318</v>
+        <v>1.328</v>
       </c>
       <c r="M34" s="21" t="n">
-        <v>1.51</v>
+        <v>1.46</v>
       </c>
       <c r="N34" s="21" t="n">
-        <v>1.626</v>
+        <v>1.651</v>
       </c>
       <c r="O34" s="21" t="n">
         <v>2.025</v>
       </c>
       <c r="P34" s="21" t="n">
-        <v>1.833</v>
+        <v>1.844</v>
       </c>
       <c r="Q34" s="21" t="n">
         <v>1.815</v>
@@ -2315,7 +2315,7 @@
         <v>27</v>
       </c>
       <c r="B35" s="20" t="n">
-        <v>1.271</v>
+        <v>1.261</v>
       </c>
       <c r="C35" s="20" t="n">
         <v>1.27</v>
@@ -2327,37 +2327,37 @@
         <v>1.43</v>
       </c>
       <c r="F35" s="21" t="n">
-        <v>1.475</v>
+        <v>1.48</v>
       </c>
       <c r="G35" s="21" t="n">
         <v>1.256</v>
       </c>
       <c r="H35" s="21" t="n">
-        <v>1.3</v>
+        <v>1.315</v>
       </c>
       <c r="I35" s="21" t="n">
         <v>1.435</v>
       </c>
       <c r="J35" s="21" t="n">
-        <v>1.23</v>
+        <v>1.24</v>
       </c>
       <c r="K35" s="21" t="n">
-        <v>1.451</v>
+        <v>1.456</v>
       </c>
       <c r="L35" s="21" t="n">
         <v>1.328</v>
       </c>
       <c r="M35" s="21" t="n">
-        <v>1.46</v>
+        <v>1.41</v>
       </c>
       <c r="N35" s="21" t="n">
-        <v>1.651</v>
+        <v>1.668</v>
       </c>
       <c r="O35" s="21" t="n">
         <v>2.025</v>
       </c>
       <c r="P35" s="21" t="n">
-        <v>1.844</v>
+        <v>1.848</v>
       </c>
       <c r="Q35" s="21" t="n">
         <v>1.815</v>
@@ -2371,7 +2371,7 @@
         <v>28</v>
       </c>
       <c r="B36" s="20" t="n">
-        <v>1.261</v>
+        <v>1.255</v>
       </c>
       <c r="C36" s="20" t="n">
         <v>1.27</v>
@@ -2380,34 +2380,34 @@
         <v>1.38</v>
       </c>
       <c r="E36" s="21" t="n">
-        <v>1.43</v>
+        <v>1.435</v>
       </c>
       <c r="F36" s="21" t="n">
-        <v>1.48</v>
+        <v>1.47</v>
       </c>
       <c r="G36" s="21" t="n">
         <v>1.256</v>
       </c>
       <c r="H36" s="21" t="n">
-        <v>1.315</v>
+        <v>1.322</v>
       </c>
       <c r="I36" s="21" t="n">
         <v>1.435</v>
       </c>
       <c r="J36" s="21" t="n">
-        <v>1.24</v>
+        <v>1.246</v>
       </c>
       <c r="K36" s="21" t="n">
         <v>1.456</v>
       </c>
       <c r="L36" s="21" t="n">
-        <v>1.328</v>
+        <v>1.322</v>
       </c>
       <c r="M36" s="21" t="n">
-        <v>1.41</v>
+        <v>1.36</v>
       </c>
       <c r="N36" s="21" t="n">
-        <v>1.668</v>
+        <v>1.679</v>
       </c>
       <c r="O36" s="21" t="n">
         <v>2.025</v>
@@ -2436,16 +2436,16 @@
         <v>1.38</v>
       </c>
       <c r="E37" s="21" t="n">
-        <v>1.435</v>
+        <v>1.465</v>
       </c>
       <c r="F37" s="21" t="n">
-        <v>1.47</v>
+        <v>1.45</v>
       </c>
       <c r="G37" s="21" t="n">
         <v>1.256</v>
       </c>
       <c r="H37" s="21" t="n">
-        <v>1.322</v>
+        <v>1.323</v>
       </c>
       <c r="I37" s="21" t="n">
         <v>1.435</v>
@@ -2457,13 +2457,13 @@
         <v>1.456</v>
       </c>
       <c r="L37" s="21" t="n">
-        <v>1.322</v>
+        <v>1.3</v>
       </c>
       <c r="M37" s="21" t="n">
-        <v>1.36</v>
+        <v>1.32</v>
       </c>
       <c r="N37" s="21" t="n">
-        <v>1.679</v>
+        <v>1.684</v>
       </c>
       <c r="O37" s="21" t="n">
         <v>2.025</v>
@@ -2472,7 +2472,7 @@
         <v>1.848</v>
       </c>
       <c r="Q37" s="21" t="n">
-        <v>1.815</v>
+        <v>1.795</v>
       </c>
       <c r="R37" s="31" t="n">
         <v>1.29</v>
@@ -2492,10 +2492,10 @@
         <v>1.38</v>
       </c>
       <c r="E38" s="21" t="n">
-        <v>1.465</v>
+        <v>1.48</v>
       </c>
       <c r="F38" s="21" t="n">
-        <v>1.45</v>
+        <v>1.438</v>
       </c>
       <c r="G38" s="21" t="n">
         <v>1.256</v>
@@ -2516,10 +2516,10 @@
         <v>1.3</v>
       </c>
       <c r="M38" s="21" t="n">
-        <v>1.32</v>
+        <v>1.291</v>
       </c>
       <c r="N38" s="21" t="n">
-        <v>1.684</v>
+        <v>1.689</v>
       </c>
       <c r="O38" s="21" t="n">
         <v>2.025</v>
@@ -2528,7 +2528,7 @@
         <v>1.848</v>
       </c>
       <c r="Q38" s="21" t="n">
-        <v>1.795</v>
+        <v>1.778</v>
       </c>
       <c r="R38" s="31" t="n">
         <v>1.285</v>
@@ -2545,13 +2545,13 @@
         <v>1.27</v>
       </c>
       <c r="D39" s="21" t="n">
-        <v>1.38</v>
+        <v>1.395</v>
       </c>
       <c r="E39" s="21" t="n">
-        <v>1.48</v>
+        <v>1.485</v>
       </c>
       <c r="F39" s="21" t="n">
-        <v>1.438</v>
+        <v>1.433</v>
       </c>
       <c r="G39" s="21" t="n">
         <v>1.256</v>
@@ -2572,19 +2572,19 @@
         <v>1.3</v>
       </c>
       <c r="M39" s="21" t="n">
-        <v>1.291</v>
+        <v>1.271</v>
       </c>
       <c r="N39" s="21" t="n">
-        <v>1.689</v>
+        <v>1.692</v>
       </c>
       <c r="O39" s="21" t="n">
-        <v>2.025</v>
+        <v>2.007</v>
       </c>
       <c r="P39" s="21" t="n">
         <v>1.848</v>
       </c>
       <c r="Q39" s="21" t="n">
-        <v>1.778</v>
+        <v>1.758</v>
       </c>
       <c r="R39" s="31" t="n">
         <v>1.285</v>
@@ -2598,16 +2598,16 @@
         <v>1.255</v>
       </c>
       <c r="C40" s="20" t="n">
-        <v>1.27</v>
+        <v>1.257</v>
       </c>
       <c r="D40" s="21" t="n">
-        <v>1.395</v>
+        <v>1.403</v>
       </c>
       <c r="E40" s="21" t="n">
         <v>1.485</v>
       </c>
       <c r="F40" s="21" t="n">
-        <v>1.433</v>
+        <v>1.423</v>
       </c>
       <c r="G40" s="21" t="n">
         <v>1.256</v>
@@ -2622,25 +2622,25 @@
         <v>1.246</v>
       </c>
       <c r="K40" s="21" t="n">
-        <v>1.456</v>
+        <v>1.465</v>
       </c>
       <c r="L40" s="21" t="n">
         <v>1.3</v>
       </c>
       <c r="M40" s="21" t="n">
-        <v>1.271</v>
+        <v>1.257</v>
       </c>
       <c r="N40" s="21" t="n">
-        <v>1.692</v>
+        <v>1.7</v>
       </c>
       <c r="O40" s="21" t="n">
-        <v>2.007</v>
+        <v>1.985</v>
       </c>
       <c r="P40" s="21" t="n">
-        <v>1.848</v>
+        <v>1.824</v>
       </c>
       <c r="Q40" s="21" t="n">
-        <v>1.758</v>
+        <v>1.73</v>
       </c>
       <c r="R40" s="31" t="n">
         <v>1.295</v>
@@ -2651,28 +2651,28 @@
         <v>33</v>
       </c>
       <c r="B41" s="20" t="n">
-        <v>1.255</v>
+        <v>1.225</v>
       </c>
       <c r="C41" s="20" t="n">
-        <v>1.257</v>
+        <v>1.235</v>
       </c>
       <c r="D41" s="21" t="n">
-        <v>1.403</v>
+        <v>1.425</v>
       </c>
       <c r="E41" s="21" t="n">
         <v>1.485</v>
       </c>
       <c r="F41" s="21" t="n">
-        <v>1.423</v>
+        <v>1.414</v>
       </c>
       <c r="G41" s="21" t="n">
-        <v>1.256</v>
+        <v>1.248</v>
       </c>
       <c r="H41" s="21" t="n">
         <v>1.323</v>
       </c>
       <c r="I41" s="21" t="n">
-        <v>1.435</v>
+        <v>1.434</v>
       </c>
       <c r="J41" s="21" t="n">
         <v>1.246</v>
@@ -2684,19 +2684,19 @@
         <v>1.3</v>
       </c>
       <c r="M41" s="21" t="n">
-        <v>1.257</v>
+        <v>1.243</v>
       </c>
       <c r="N41" s="21" t="n">
-        <v>1.7</v>
+        <v>1.707</v>
       </c>
       <c r="O41" s="21" t="n">
-        <v>1.985</v>
+        <v>1.957</v>
       </c>
       <c r="P41" s="21" t="n">
         <v>1.824</v>
       </c>
       <c r="Q41" s="21" t="n">
-        <v>1.73</v>
+        <v>1.701</v>
       </c>
       <c r="R41" s="31" t="n">
         <v>1.325</v>
@@ -2707,28 +2707,28 @@
         <v>34</v>
       </c>
       <c r="B42" s="20" t="n">
-        <v>1.225</v>
+        <v>1.19</v>
       </c>
       <c r="C42" s="20" t="n">
-        <v>1.235</v>
+        <v>1.223</v>
       </c>
       <c r="D42" s="21" t="n">
-        <v>1.425</v>
+        <v>1.45</v>
       </c>
       <c r="E42" s="21" t="n">
-        <v>1.485</v>
+        <v>1.513</v>
       </c>
       <c r="F42" s="21" t="n">
-        <v>1.414</v>
+        <v>1.4</v>
       </c>
       <c r="G42" s="21" t="n">
-        <v>1.248</v>
+        <v>1.24</v>
       </c>
       <c r="H42" s="21" t="n">
-        <v>1.323</v>
+        <v>1.321</v>
       </c>
       <c r="I42" s="21" t="n">
-        <v>1.434</v>
+        <v>1.424</v>
       </c>
       <c r="J42" s="21" t="n">
         <v>1.246</v>
@@ -2740,19 +2740,19 @@
         <v>1.3</v>
       </c>
       <c r="M42" s="21" t="n">
-        <v>1.243</v>
+        <v>1.233</v>
       </c>
       <c r="N42" s="21" t="n">
-        <v>1.707</v>
+        <v>1.714</v>
       </c>
       <c r="O42" s="21" t="n">
-        <v>1.957</v>
+        <v>1.93</v>
       </c>
       <c r="P42" s="21" t="n">
-        <v>1.824</v>
+        <v>1.799</v>
       </c>
       <c r="Q42" s="21" t="n">
-        <v>1.701</v>
+        <v>1.671</v>
       </c>
       <c r="R42" s="31" t="n">
         <v>1.35</v>
@@ -2763,31 +2763,31 @@
         <v>35</v>
       </c>
       <c r="B43" s="20" t="n">
-        <v>1.19</v>
+        <v>1.142</v>
       </c>
       <c r="C43" s="20" t="n">
         <v>1.223</v>
       </c>
       <c r="D43" s="21" t="n">
-        <v>1.45</v>
+        <v>1.475</v>
       </c>
       <c r="E43" s="21" t="n">
-        <v>1.513</v>
+        <v>1.533</v>
       </c>
       <c r="F43" s="21" t="n">
-        <v>1.4</v>
+        <v>1.38</v>
       </c>
       <c r="G43" s="21" t="n">
-        <v>1.24</v>
+        <v>1.227</v>
       </c>
       <c r="H43" s="21" t="n">
-        <v>1.321</v>
+        <v>1.32</v>
       </c>
       <c r="I43" s="21" t="n">
-        <v>1.424</v>
+        <v>1.41</v>
       </c>
       <c r="J43" s="21" t="n">
-        <v>1.246</v>
+        <v>1.245</v>
       </c>
       <c r="K43" s="21" t="n">
         <v>1.465</v>
@@ -2796,19 +2796,19 @@
         <v>1.3</v>
       </c>
       <c r="M43" s="21" t="n">
-        <v>1.233</v>
+        <v>1.215</v>
       </c>
       <c r="N43" s="21" t="n">
-        <v>1.714</v>
+        <v>1.719</v>
       </c>
       <c r="O43" s="21" t="n">
-        <v>1.93</v>
+        <v>1.905</v>
       </c>
       <c r="P43" s="21" t="n">
-        <v>1.799</v>
+        <v>1.774</v>
       </c>
       <c r="Q43" s="21" t="n">
-        <v>1.671</v>
+        <v>1.643</v>
       </c>
       <c r="R43" s="31" t="n">
         <v>1.36</v>
@@ -2819,31 +2819,31 @@
         <v>36</v>
       </c>
       <c r="B44" s="20" t="n">
-        <v>1.142</v>
+        <v>1.112</v>
       </c>
       <c r="C44" s="20" t="n">
         <v>1.223</v>
       </c>
       <c r="D44" s="21" t="n">
-        <v>1.475</v>
+        <v>1.49</v>
       </c>
       <c r="E44" s="21" t="n">
         <v>1.533</v>
       </c>
       <c r="F44" s="21" t="n">
-        <v>1.38</v>
+        <v>1.358</v>
       </c>
       <c r="G44" s="21" t="n">
-        <v>1.227</v>
+        <v>1.217</v>
       </c>
       <c r="H44" s="21" t="n">
         <v>1.32</v>
       </c>
       <c r="I44" s="21" t="n">
-        <v>1.41</v>
+        <v>1.389</v>
       </c>
       <c r="J44" s="21" t="n">
-        <v>1.245</v>
+        <v>1.225</v>
       </c>
       <c r="K44" s="21" t="n">
         <v>1.465</v>
@@ -2852,19 +2852,19 @@
         <v>1.3</v>
       </c>
       <c r="M44" s="21" t="n">
-        <v>1.215</v>
+        <v>1.197</v>
       </c>
       <c r="N44" s="21" t="n">
-        <v>1.719</v>
+        <v>1.722</v>
       </c>
       <c r="O44" s="21" t="n">
-        <v>1.905</v>
+        <v>1.883</v>
       </c>
       <c r="P44" s="21" t="n">
-        <v>1.774</v>
+        <v>1.752</v>
       </c>
       <c r="Q44" s="21" t="n">
-        <v>1.643</v>
+        <v>1.617</v>
       </c>
       <c r="R44" s="31" t="n">
         <v>1.363</v>
@@ -2875,7 +2875,7 @@
         <v>37</v>
       </c>
       <c r="B45" s="23" t="n">
-        <v>1.112</v>
+        <v>1.102</v>
       </c>
       <c r="C45" s="20" t="n">
         <v>1.223</v>
@@ -2884,22 +2884,22 @@
         <v>1.49</v>
       </c>
       <c r="E45" s="21" t="n">
-        <v>1.533</v>
+        <v>1.503</v>
       </c>
       <c r="F45" s="21" t="n">
-        <v>1.358</v>
+        <v>1.325</v>
       </c>
       <c r="G45" s="21" t="n">
-        <v>1.217</v>
+        <v>1.205</v>
       </c>
       <c r="H45" s="21" t="n">
-        <v>1.32</v>
+        <v>1.325</v>
       </c>
       <c r="I45" s="21" t="n">
-        <v>1.389</v>
+        <v>1.34</v>
       </c>
       <c r="J45" s="21" t="n">
-        <v>1.225</v>
+        <v>1.2</v>
       </c>
       <c r="K45" s="21" t="n">
         <v>1.465</v>
@@ -2908,19 +2908,19 @@
         <v>1.3</v>
       </c>
       <c r="M45" s="21" t="n">
-        <v>1.197</v>
+        <v>1.173</v>
       </c>
       <c r="N45" s="21" t="n">
         <v>1.722</v>
       </c>
       <c r="O45" s="21" t="n">
-        <v>1.883</v>
+        <v>1.858</v>
       </c>
       <c r="P45" s="21" t="n">
-        <v>1.752</v>
+        <v>1.729</v>
       </c>
       <c r="Q45" s="21" t="n">
-        <v>1.617</v>
+        <v>1.587</v>
       </c>
       <c r="R45" s="31" t="n">
         <v>1.365</v>
@@ -2931,7 +2931,7 @@
         <v>38</v>
       </c>
       <c r="B46" s="20" t="n">
-        <v>1.102</v>
+        <v>1.076</v>
       </c>
       <c r="C46" s="20" t="n">
         <v>1.223</v>
@@ -2940,43 +2940,43 @@
         <v>1.49</v>
       </c>
       <c r="E46" s="21" t="n">
-        <v>1.503</v>
+        <v>1.47</v>
       </c>
       <c r="F46" s="21" t="n">
-        <v>1.325</v>
+        <v>1.267</v>
       </c>
       <c r="G46" s="21" t="n">
-        <v>1.205</v>
+        <v>1.185</v>
       </c>
       <c r="H46" s="21" t="n">
         <v>1.325</v>
       </c>
       <c r="I46" s="21" t="n">
-        <v>1.34</v>
+        <v>1.293</v>
       </c>
       <c r="J46" s="21" t="n">
-        <v>1.2</v>
+        <v>1.17</v>
       </c>
       <c r="K46" s="21" t="n">
         <v>1.465</v>
       </c>
       <c r="L46" s="21" t="n">
-        <v>1.3</v>
+        <v>1.296</v>
       </c>
       <c r="M46" s="21" t="n">
-        <v>1.173</v>
+        <v>1.147</v>
       </c>
       <c r="N46" s="21" t="n">
         <v>1.722</v>
       </c>
       <c r="O46" s="21" t="n">
-        <v>1.858</v>
+        <v>1.829</v>
       </c>
       <c r="P46" s="21" t="n">
-        <v>1.729</v>
+        <v>1.704</v>
       </c>
       <c r="Q46" s="21" t="n">
-        <v>1.587</v>
+        <v>1.552</v>
       </c>
       <c r="R46" s="31" t="n">
         <v>1.34</v>
@@ -2987,7 +2987,7 @@
         <v>39</v>
       </c>
       <c r="B47" s="20" t="n">
-        <v>1.076</v>
+        <v>1.04</v>
       </c>
       <c r="C47" s="23" t="n">
         <v>1.223</v>
@@ -2996,43 +2996,43 @@
         <v>1.49</v>
       </c>
       <c r="E47" s="21" t="n">
-        <v>1.47</v>
+        <v>1.432</v>
       </c>
       <c r="F47" s="21" t="n">
-        <v>1.267</v>
+        <v>1.212</v>
       </c>
       <c r="G47" s="21" t="n">
-        <v>1.185</v>
+        <v>1.155</v>
       </c>
       <c r="H47" s="21" t="n">
-        <v>1.325</v>
+        <v>1.3</v>
       </c>
       <c r="I47" s="21" t="n">
-        <v>1.293</v>
+        <v>1.24</v>
       </c>
       <c r="J47" s="21" t="n">
-        <v>1.17</v>
+        <v>1.144</v>
       </c>
       <c r="K47" s="21" t="n">
-        <v>1.465</v>
+        <v>1.458</v>
       </c>
       <c r="L47" s="21" t="n">
         <v>1.296</v>
       </c>
       <c r="M47" s="21" t="n">
-        <v>1.147</v>
+        <v>1.114</v>
       </c>
       <c r="N47" s="21" t="n">
         <v>1.722</v>
       </c>
       <c r="O47" s="21" t="n">
-        <v>1.829</v>
+        <v>1.803</v>
       </c>
       <c r="P47" s="21" t="n">
-        <v>1.704</v>
+        <v>1.679</v>
       </c>
       <c r="Q47" s="21" t="n">
-        <v>1.552</v>
+        <v>1.52</v>
       </c>
       <c r="R47" s="22" t="n">
         <v>1.315</v>
@@ -3043,52 +3043,52 @@
         <v>40</v>
       </c>
       <c r="B48" s="20" t="n">
-        <v>1.04</v>
+        <v>1.018</v>
       </c>
       <c r="C48" s="23" t="n">
-        <v>1.223</v>
+        <v>1.208</v>
       </c>
       <c r="D48" s="21" t="n">
         <v>1.49</v>
       </c>
       <c r="E48" s="21" t="n">
-        <v>1.432</v>
+        <v>1.404</v>
       </c>
       <c r="F48" s="21" t="n">
-        <v>1.212</v>
+        <v>1.155</v>
       </c>
       <c r="G48" s="21" t="n">
-        <v>1.155</v>
+        <v>1.124</v>
       </c>
       <c r="H48" s="21" t="n">
-        <v>1.3</v>
+        <v>1.262</v>
       </c>
       <c r="I48" s="21" t="n">
-        <v>1.24</v>
+        <v>1.183</v>
       </c>
       <c r="J48" s="21" t="n">
-        <v>1.144</v>
+        <v>1.124</v>
       </c>
       <c r="K48" s="21" t="n">
-        <v>1.458</v>
+        <v>1.451</v>
       </c>
       <c r="L48" s="21" t="n">
         <v>1.296</v>
       </c>
       <c r="M48" s="21" t="n">
-        <v>1.114</v>
+        <v>1.079</v>
       </c>
       <c r="N48" s="21" t="n">
         <v>1.722</v>
       </c>
       <c r="O48" s="21" t="n">
-        <v>1.803</v>
+        <v>1.774</v>
       </c>
       <c r="P48" s="21" t="n">
-        <v>1.679</v>
+        <v>1.655</v>
       </c>
       <c r="Q48" s="21" t="n">
-        <v>1.52</v>
+        <v>1.491</v>
       </c>
       <c r="R48" s="21" t="n">
         <v>1.295</v>
@@ -3099,52 +3099,52 @@
         <v>41</v>
       </c>
       <c r="B49" s="20" t="n">
-        <v>1.018</v>
+        <v>1.014</v>
       </c>
       <c r="C49" s="20" t="n">
-        <v>1.208</v>
+        <v>1.2</v>
       </c>
       <c r="D49" s="21" t="n">
-        <v>1.49</v>
+        <v>1.48</v>
       </c>
       <c r="E49" s="21" t="n">
-        <v>1.404</v>
+        <v>1.383</v>
       </c>
       <c r="F49" s="21" t="n">
-        <v>1.155</v>
+        <v>1.12</v>
       </c>
       <c r="G49" s="21" t="n">
-        <v>1.124</v>
+        <v>1.1</v>
       </c>
       <c r="H49" s="21" t="n">
-        <v>1.262</v>
+        <v>1.217</v>
       </c>
       <c r="I49" s="21" t="n">
-        <v>1.183</v>
+        <v>1.137</v>
       </c>
       <c r="J49" s="21" t="n">
-        <v>1.124</v>
+        <v>1.1</v>
       </c>
       <c r="K49" s="21" t="n">
-        <v>1.451</v>
+        <v>1.44</v>
       </c>
       <c r="L49" s="21" t="n">
         <v>1.296</v>
       </c>
       <c r="M49" s="21" t="n">
-        <v>1.079</v>
+        <v>1.051</v>
       </c>
       <c r="N49" s="21" t="n">
-        <v>1.722</v>
+        <v>1.717</v>
       </c>
       <c r="O49" s="21" t="n">
-        <v>1.774</v>
+        <v>1.739</v>
       </c>
       <c r="P49" s="21" t="n">
-        <v>1.655</v>
+        <v>1.633</v>
       </c>
       <c r="Q49" s="21" t="n">
-        <v>1.491</v>
+        <v>1.445</v>
       </c>
       <c r="R49" s="21" t="n"/>
     </row>
@@ -3156,49 +3156,49 @@
         <v>1.014</v>
       </c>
       <c r="C50" s="20" t="n">
-        <v>1.2</v>
+        <v>1.195</v>
       </c>
       <c r="D50" s="21" t="n">
-        <v>1.48</v>
+        <v>1.46</v>
       </c>
       <c r="E50" s="21" t="n">
-        <v>1.383</v>
+        <v>1.371</v>
       </c>
       <c r="F50" s="21" t="n">
-        <v>1.12</v>
+        <v>1.1</v>
       </c>
       <c r="G50" s="21" t="n">
-        <v>1.1</v>
+        <v>1.075</v>
       </c>
       <c r="H50" s="21" t="n">
-        <v>1.217</v>
+        <v>1.18</v>
       </c>
       <c r="I50" s="21" t="n">
-        <v>1.137</v>
+        <v>1.105</v>
       </c>
       <c r="J50" s="21" t="n">
-        <v>1.1</v>
+        <v>1.076</v>
       </c>
       <c r="K50" s="21" t="n">
-        <v>1.44</v>
+        <v>1.435</v>
       </c>
       <c r="L50" s="21" t="n">
-        <v>1.296</v>
+        <v>1.293</v>
       </c>
       <c r="M50" s="21" t="n">
-        <v>1.051</v>
+        <v>1.032</v>
       </c>
       <c r="N50" s="21" t="n">
-        <v>1.717</v>
+        <v>1.701</v>
       </c>
       <c r="O50" s="21" t="n">
-        <v>1.739</v>
+        <v>1.707</v>
       </c>
       <c r="P50" s="21" t="n">
-        <v>1.633</v>
+        <v>1.611</v>
       </c>
       <c r="Q50" s="21" t="n">
-        <v>1.445</v>
+        <v>1.411</v>
       </c>
       <c r="R50" s="21" t="n"/>
     </row>
@@ -3207,52 +3207,52 @@
         <v>43</v>
       </c>
       <c r="B51" s="20" t="n">
-        <v>1.014</v>
+        <v>1.013</v>
       </c>
       <c r="C51" s="20" t="n">
-        <v>1.195</v>
+        <v>1.19</v>
       </c>
       <c r="D51" s="21" t="n">
-        <v>1.46</v>
+        <v>1.42</v>
       </c>
       <c r="E51" s="21" t="n">
-        <v>1.371</v>
+        <v>1.368</v>
       </c>
       <c r="F51" s="21" t="n">
-        <v>1.1</v>
+        <v>1.09</v>
       </c>
       <c r="G51" s="21" t="n">
+        <v>1.052</v>
+      </c>
+      <c r="H51" s="21" t="n">
+        <v>1.16</v>
+      </c>
+      <c r="I51" s="21" t="n">
         <v>1.075</v>
       </c>
-      <c r="H51" s="21" t="n">
-        <v>1.18</v>
-      </c>
-      <c r="I51" s="21" t="n">
-        <v>1.105</v>
-      </c>
       <c r="J51" s="21" t="n">
-        <v>1.076</v>
+        <v>1.056</v>
       </c>
       <c r="K51" s="21" t="n">
-        <v>1.435</v>
+        <v>1.428</v>
       </c>
       <c r="L51" s="21" t="n">
-        <v>1.293</v>
+        <v>1.283</v>
       </c>
       <c r="M51" s="21" t="n">
-        <v>1.032</v>
+        <v>1.023</v>
       </c>
       <c r="N51" s="21" t="n">
-        <v>1.701</v>
+        <v>1.678</v>
       </c>
       <c r="O51" s="21" t="n">
-        <v>1.707</v>
+        <v>1.68</v>
       </c>
       <c r="P51" s="21" t="n">
-        <v>1.611</v>
+        <v>1.587</v>
       </c>
       <c r="Q51" s="21" t="n">
-        <v>1.411</v>
+        <v>1.385</v>
       </c>
       <c r="R51" s="21" t="n"/>
     </row>
@@ -3261,52 +3261,52 @@
         <v>44</v>
       </c>
       <c r="B52" s="20" t="n">
-        <v>1.013</v>
+        <v>1.014</v>
       </c>
       <c r="C52" s="20" t="n">
         <v>1.19</v>
       </c>
       <c r="D52" s="21" t="n">
-        <v>1.42</v>
+        <v>1.392</v>
       </c>
       <c r="E52" s="21" t="n">
-        <v>1.368</v>
+        <v>1.335</v>
       </c>
       <c r="F52" s="21" t="n">
         <v>1.09</v>
       </c>
       <c r="G52" s="21" t="n">
-        <v>1.052</v>
+        <v>1.029</v>
       </c>
       <c r="H52" s="21" t="n">
-        <v>1.16</v>
+        <v>1.143</v>
       </c>
       <c r="I52" s="21" t="n">
-        <v>1.075</v>
+        <v>1.055</v>
       </c>
       <c r="J52" s="21" t="n">
-        <v>1.056</v>
+        <v>1.046</v>
       </c>
       <c r="K52" s="21" t="n">
-        <v>1.428</v>
+        <v>1.425</v>
       </c>
       <c r="L52" s="21" t="n">
-        <v>1.283</v>
+        <v>1.264</v>
       </c>
       <c r="M52" s="21" t="n">
-        <v>1.023</v>
+        <v>1.02</v>
       </c>
       <c r="N52" s="21" t="n">
-        <v>1.678</v>
+        <v>1.659</v>
       </c>
       <c r="O52" s="21" t="n">
-        <v>1.68</v>
+        <v>1.658</v>
       </c>
       <c r="P52" s="21" t="n">
-        <v>1.587</v>
+        <v>1.571</v>
       </c>
       <c r="Q52" s="21" t="n">
-        <v>1.385</v>
+        <v>1.369</v>
       </c>
       <c r="R52" s="21" t="n"/>
     </row>
@@ -3321,46 +3321,46 @@
         <v>1.19</v>
       </c>
       <c r="D53" s="21" t="n">
-        <v>1.392</v>
+        <v>1.368</v>
       </c>
       <c r="E53" s="21" t="n">
-        <v>1.335</v>
+        <v>1.295</v>
       </c>
       <c r="F53" s="21" t="n">
         <v>1.09</v>
       </c>
       <c r="G53" s="21" t="n">
-        <v>1.029</v>
+        <v>1.007</v>
       </c>
       <c r="H53" s="21" t="n">
-        <v>1.143</v>
+        <v>1.132</v>
       </c>
       <c r="I53" s="21" t="n">
-        <v>1.055</v>
+        <v>1.038</v>
       </c>
       <c r="J53" s="21" t="n">
-        <v>1.046</v>
+        <v>1.041</v>
       </c>
       <c r="K53" s="21" t="n">
         <v>1.425</v>
       </c>
       <c r="L53" s="21" t="n">
-        <v>1.264</v>
+        <v>1.239</v>
       </c>
       <c r="M53" s="21" t="n">
         <v>1.02</v>
       </c>
       <c r="N53" s="21" t="n">
-        <v>1.659</v>
+        <v>1.645</v>
       </c>
       <c r="O53" s="21" t="n">
-        <v>1.658</v>
+        <v>1.641</v>
       </c>
       <c r="P53" s="21" t="n">
-        <v>1.571</v>
+        <v>1.565</v>
       </c>
       <c r="Q53" s="21" t="n">
-        <v>1.369</v>
+        <v>1.359</v>
       </c>
       <c r="R53" s="21" t="n"/>
     </row>
@@ -3372,49 +3372,49 @@
         <v>1.014</v>
       </c>
       <c r="C54" s="20" t="n">
-        <v>1.19</v>
+        <v>1.185</v>
       </c>
       <c r="D54" s="21" t="n">
-        <v>1.368</v>
+        <v>1.357</v>
       </c>
       <c r="E54" s="21" t="n">
-        <v>1.295</v>
+        <v>1.29</v>
       </c>
       <c r="F54" s="21" t="n">
         <v>1.09</v>
       </c>
       <c r="G54" s="21" t="n">
-        <v>1.007</v>
+        <v>0.992</v>
       </c>
       <c r="H54" s="21" t="n">
         <v>1.132</v>
       </c>
       <c r="I54" s="21" t="n">
+        <v>1.028</v>
+      </c>
+      <c r="J54" s="21" t="n">
         <v>1.038</v>
       </c>
-      <c r="J54" s="21" t="n">
-        <v>1.041</v>
-      </c>
       <c r="K54" s="21" t="n">
-        <v>1.425</v>
+        <v>1.428</v>
       </c>
       <c r="L54" s="21" t="n">
-        <v>1.239</v>
+        <v>1.204</v>
       </c>
       <c r="M54" s="21" t="n">
         <v>1.02</v>
       </c>
       <c r="N54" s="21" t="n">
-        <v>1.645</v>
+        <v>1.64</v>
       </c>
       <c r="O54" s="21" t="n">
-        <v>1.641</v>
+        <v>1.636</v>
       </c>
       <c r="P54" s="21" t="n">
         <v>1.565</v>
       </c>
       <c r="Q54" s="21" t="n">
-        <v>1.359</v>
+        <v>1.354</v>
       </c>
       <c r="R54" s="21" t="n"/>
     </row>
@@ -3426,10 +3426,10 @@
         <v>1.014</v>
       </c>
       <c r="C55" s="20" t="n">
-        <v>1.185</v>
+        <v>1.182</v>
       </c>
       <c r="D55" s="21" t="n">
-        <v>1.357</v>
+        <v>1.342</v>
       </c>
       <c r="E55" s="21" t="n">
         <v>1.29</v>
@@ -3438,7 +3438,7 @@
         <v>1.09</v>
       </c>
       <c r="G55" s="21" t="n">
-        <v>0.992</v>
+        <v>0.975</v>
       </c>
       <c r="H55" s="21" t="n">
         <v>1.132</v>
@@ -3450,10 +3450,10 @@
         <v>1.038</v>
       </c>
       <c r="K55" s="21" t="n">
-        <v>1.428</v>
+        <v>1.454</v>
       </c>
       <c r="L55" s="21" t="n">
-        <v>1.204</v>
+        <v>1.165</v>
       </c>
       <c r="M55" s="21" t="n">
         <v>1.02</v>
@@ -3462,13 +3462,13 @@
         <v>1.64</v>
       </c>
       <c r="O55" s="21" t="n">
-        <v>1.636</v>
+        <v>1.634</v>
       </c>
       <c r="P55" s="21" t="n">
         <v>1.565</v>
       </c>
       <c r="Q55" s="21" t="n">
-        <v>1.354</v>
+        <v>1.314</v>
       </c>
       <c r="R55" s="21" t="n"/>
     </row>
@@ -3480,19 +3480,19 @@
         <v>1.014</v>
       </c>
       <c r="C56" s="20" t="n">
-        <v>1.182</v>
+        <v>1.177</v>
       </c>
       <c r="D56" s="21" t="n">
-        <v>1.342</v>
+        <v>1.328</v>
       </c>
       <c r="E56" s="21" t="n">
         <v>1.29</v>
       </c>
       <c r="F56" s="21" t="n">
-        <v>1.09</v>
+        <v>1.08</v>
       </c>
       <c r="G56" s="21" t="n">
-        <v>0.975</v>
+        <v>0.963</v>
       </c>
       <c r="H56" s="21" t="n">
         <v>1.132</v>
@@ -3504,10 +3504,10 @@
         <v>1.038</v>
       </c>
       <c r="K56" s="21" t="n">
-        <v>1.454</v>
+        <v>1.488</v>
       </c>
       <c r="L56" s="21" t="n">
-        <v>1.165</v>
+        <v>1.126</v>
       </c>
       <c r="M56" s="21" t="n">
         <v>1.02</v>
@@ -3522,7 +3522,7 @@
         <v>1.565</v>
       </c>
       <c r="Q56" s="21" t="n">
-        <v>1.314</v>
+        <v>1.3</v>
       </c>
       <c r="R56" s="21" t="n"/>
     </row>
@@ -3531,22 +3531,22 @@
         <v>49</v>
       </c>
       <c r="B57" s="20" t="n">
-        <v>1.014</v>
+        <v>1.026</v>
       </c>
       <c r="C57" s="20" t="n">
         <v>1.177</v>
       </c>
       <c r="D57" s="21" t="n">
-        <v>1.328</v>
+        <v>1.315</v>
       </c>
       <c r="E57" s="21" t="n">
-        <v>1.29</v>
+        <v>1.295</v>
       </c>
       <c r="F57" s="21" t="n">
-        <v>1.08</v>
+        <v>1.055</v>
       </c>
       <c r="G57" s="21" t="n">
-        <v>0.963</v>
+        <v>0.953</v>
       </c>
       <c r="H57" s="21" t="n">
         <v>1.132</v>
@@ -3558,16 +3558,16 @@
         <v>1.038</v>
       </c>
       <c r="K57" s="21" t="n">
-        <v>1.488</v>
+        <v>1.505</v>
       </c>
       <c r="L57" s="21" t="n">
-        <v>1.126</v>
+        <v>1.106</v>
       </c>
       <c r="M57" s="21" t="n">
         <v>1.02</v>
       </c>
       <c r="N57" s="21" t="n">
-        <v>1.64</v>
+        <v>1.645</v>
       </c>
       <c r="O57" s="21" t="n">
         <v>1.634</v>
@@ -3576,7 +3576,7 @@
         <v>1.565</v>
       </c>
       <c r="Q57" s="21" t="n">
-        <v>1.2</v>
+        <v>1.1</v>
       </c>
       <c r="R57" s="21" t="n"/>
     </row>
@@ -3585,22 +3585,22 @@
         <v>50</v>
       </c>
       <c r="B58" s="20" t="n">
-        <v>1.026</v>
+        <v>1.03</v>
       </c>
       <c r="C58" s="20" t="n">
-        <v>1.177</v>
+        <v>1.162</v>
       </c>
       <c r="D58" s="21" t="n">
-        <v>1.315</v>
+        <v>1.31</v>
       </c>
       <c r="E58" s="21" t="n">
-        <v>1.295</v>
+        <v>1.29</v>
       </c>
       <c r="F58" s="21" t="n">
-        <v>1.055</v>
+        <v>1.045</v>
       </c>
       <c r="G58" s="21" t="n">
-        <v>0.953</v>
+        <v>0.95</v>
       </c>
       <c r="H58" s="21" t="n">
         <v>1.132</v>
@@ -3612,10 +3612,10 @@
         <v>1.038</v>
       </c>
       <c r="K58" s="21" t="n">
-        <v>1.505</v>
+        <v>1.508</v>
       </c>
       <c r="L58" s="21" t="n">
-        <v>1.106</v>
+        <v>1.098</v>
       </c>
       <c r="M58" s="21" t="n">
         <v>1.02</v>
@@ -3630,7 +3630,7 @@
         <v>1.565</v>
       </c>
       <c r="Q58" s="21" t="n">
-        <v>1.1</v>
+        <v>1.04</v>
       </c>
       <c r="R58" s="21" t="n"/>
     </row>
@@ -3642,34 +3642,34 @@
         <v>1.03</v>
       </c>
       <c r="C59" s="20" t="n">
-        <v>1.162</v>
+        <v>1.147</v>
       </c>
       <c r="D59" s="21" t="n">
-        <v>1.31</v>
+        <v>1.305</v>
       </c>
       <c r="E59" s="21" t="n">
-        <v>1.29</v>
+        <v>1.253</v>
       </c>
       <c r="F59" s="21" t="n">
-        <v>1.045</v>
+        <v>1.043</v>
       </c>
       <c r="G59" s="21" t="n">
-        <v>0.95</v>
+        <v>0.947</v>
       </c>
       <c r="H59" s="21" t="n">
-        <v>1.132</v>
+        <v>1.129</v>
       </c>
       <c r="I59" s="21" t="n">
-        <v>1.028</v>
+        <v>1.015</v>
       </c>
       <c r="J59" s="21" t="n">
         <v>1.038</v>
       </c>
       <c r="K59" s="21" t="n">
-        <v>1.508</v>
+        <v>1.49</v>
       </c>
       <c r="L59" s="21" t="n">
-        <v>1.098</v>
+        <v>1.096</v>
       </c>
       <c r="M59" s="21" t="n">
         <v>1.02</v>
@@ -3696,10 +3696,10 @@
         <v>1.03</v>
       </c>
       <c r="C60" s="20" t="n">
-        <v>1.147</v>
+        <v>1.127</v>
       </c>
       <c r="D60" s="21" t="n">
-        <v>1.305</v>
+        <v>1.303</v>
       </c>
       <c r="E60" s="21" t="n">
         <v>1.253</v>

</xml_diff>